<commit_message>
Remove Blueground short-term sublet; scope = 2025/2026 NYC rentals & purchases only
515 E 86th #202 (Blueground) was a 6-week furnished sublet, not a
long-term rental or purchase search. List is now 7 apartments.

https://claude.ai/code/session_01MbNWBgH9MLGMgH6Ytb3ovm
</commit_message>
<xml_diff>
--- a/NYC_Apartment_Tracker.xlsx
+++ b/NYC_Apartment_Tracker.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -951,55 +951,6 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>515 East 86th Street, New York, NY 10028</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>202</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>https://streeteasy.com/for-rent/listing/515-east-86th-street</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Rent</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Jarvis / Blueground Sales (Blueground at Convivium)</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>sales-nyc@theblueground.com</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>May 2025</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>Short-term furnished rental via Blueground at Convivium. Available May 20 – Jun 30, 2025. Dynamic pricing. Inquiry via StreetEasy May 2025.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <hyperlinks>
@@ -1010,7 +961,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebuild tracker: 2026-only scope, add rental inquiries, date+time showing, date contacted column
- Removed all 2025 apartments (165 E 72nd #12J, 310 E 70th #10E, 239 E 79th #13L, 420 E 80th #PHD)
- Kept 3 purchase listings (200 E 90th #16E, 10 East End Ave #18A, 520 E 72nd #PHC)
- Added 4 new 2026 rental inquiry entries found in Gmail sent/StreetEasy confirmations:
  265 E 66th #34B (showing May 31 12pm), 240 E 82nd #18B (scheduling),
  345 E 80th #27B (circle back), 170 E 87th #W4H (awaiting response)
- Added 'Date Contacted' column
- Date of Showing now includes date AND time where known
- New status values: Showing Scheduled, Contacted – Scheduling,
  Contacted – Awaiting Response, Contacted – Circle Back When Ready
- New blue row color for 'Contacted' rental rows
- Updated How to Use tab with full status/colour key

https://claude.ai/code/session_01MbNWBgH9MLGMgH6Ytb3ovm
</commit_message>
<xml_diff>
--- a/NYC_Apartment_Tracker.xlsx
+++ b/NYC_Apartment_Tracker.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to Use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Apartment Tracker'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Apartment Tracker'!$A$1:$L$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -69,12 +69,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -516,11 +516,12 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -566,21 +567,26 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Date Contacted</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Date of Showing</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="65" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>200 East 90th Street, New York, NY 10128</t>
@@ -623,21 +629,26 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>May 3, 2026</t>
+          <t>Jan 2026</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
+          <t>May 3, 2026 at 11:00 AM</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
           <t>Active – Negotiating</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Co-op. Asking reduced from $1.25M → $1.15M. Offer $1,020,000; seller countered at $1,125,000. High floor, East River views. Buyer's broker: Saree Ptak (sareerptak@gmail.com).</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="65" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>10 East End Avenue, New York, NY 10028</t>
@@ -680,21 +691,26 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Jan 11, 2026</t>
+          <t>Jan 2026</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
+          <t>Jan 12, 2026 at 9:45 AM</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
           <t>Under Contract</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Co-op. Estate sale (Estate of Tuppatsch). Agreed price $1,150,000. Contract in progress with attorney Andy Cutler. Court action (estate) adjourned to 5/5/26. Chase mortgage (7yr ARM 4.750%). Buyer's broker: Saree Ptak (sareerptak@gmail.com).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="65" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>520 East 72nd Street, New York, NY 10021</t>
@@ -729,193 +745,205 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
           <t>Jan 11, 2026</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Inquired</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Co-op. 30% down building; no W/D in unit; no investors allowed. DTI &lt; 30% required. 2% buyer's agent commission. Buyer's broker: Saree Ptak (sareerptak@gmail.com).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="65" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>165 East 72nd Street, New York, NY 10021</t>
+          <t>265 East 66th Street, New York, NY 10065</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>12J</t>
+          <t>34B</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>https://streeteasy.com/building/165-east-72nd-street-new_york</t>
+          <t>https://streeteasy.com/building/265-east-66th-street-new_york</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Purchase</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr"/>
       <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Elisabeth Quick (Serhant)</t>
+          <t>Joseph George (MNS Real Estate)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>quick@serhant.com</t>
+          <t>jgj@mns.com</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Dec 2025</t>
+          <t>May 25, 2026</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Passed – renovation cost too high. Buyer's broker: Saree Ptak (sareerptak@gmail.com).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>310 East 70th Street, New York, NY 10021</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>10E</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>https://streeteasy.com/building/310-east-70th-street-new_york</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Purchase</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>$1,395,000</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>$1,225,000</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Jesse Klein (Compass)</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>jesse.klein@compass.com</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>Nov 5, 2025</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>Co-op. Asking reduced from ~$1.45M → $1,395,000. Offer $1,225,000; seller countered at $1,395,000. Subletting policy: 2 out of 5 years. Buyer's broker: Saree Ptak (sareerptak@gmail.com).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>239 East 79th Street, New York, NY 10075</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>13L</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>https://streeteasy.com/building/239-east-79th-street-new_york</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Purchase</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>$1,375,000</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Roger J. Gillen (Brown Harris Stevens)</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>RGillen@bhsusa.com</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Nov 2025</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>Co-op. Asking $1,375,000. Passed – major renovation needed (2011 updates outdated). Broker rejected low offer. Buyer's broker: Saree Ptak (sareerptak@gmail.com).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+          <t>May 31, 2026 at 12:00 PM</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Showing Scheduled</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Rental inquiry sent May 25, 2026 (via Harley's StreetEasy account). Showing confirmed: Sunday May 31, 2026 at 12:00 PM ET. Contact: Joseph George, MNS Real Estate (jgj@mns.com).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="65" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>240 East 82nd Street, New York, NY 10028</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>18B</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>https://streeteasy.com/building/240-east-82nd-street-new_york</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>$7,000/mo</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Tomi Bicanic (Citywide Apts)</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>tomi.bicanic@citywideapts.com</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>May 24, 2026</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>TBD – Sat May 30/31 requested</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>Contacted – Scheduling</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>StreetEasy inquiry sent May 24, 2026. $7,000/mo. Celine requested Saturday tour (out of town until Sat). Contact: Tomi Bicanic, Citywide Apts (tomi.bicanic@citywideapts.com).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="65" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>345 East 80th Street, New York, NY 10075</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>27B</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>https://streeteasy.com/building/345-east-80th-street-new_york</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr"/>
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Anis (PocketBroker)</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>anis@pocketbroker.com</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>May 24, 2026</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>Contacted – Circle Back When Ready</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>StreetEasy inquiry sent May 24, 2026. Broker replied: "Enjoy your travels. Circle back to us then." Also cc: diana@pocketbroker.com. Follow up when back in town.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="65" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>420 East 80th Street, New York, NY 10075</t>
+          <t>170 East 87th Street, New York, NY 10128</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>PHD</t>
+          <t>W4H</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>https://streeteasy.com/for-rent/listing/420-east-80th-street</t>
+          <t>https://streeteasy.com/building/170-east-87th-street-new_york</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -925,34 +953,31 @@
       </c>
       <c r="E8" s="9" t="inlineStr"/>
       <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Maria Skovranova (The Ashford NYC)</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>Leasing_Office-theashfordnyc@knck.io</t>
-        </is>
-      </c>
+      <c r="G8" s="8" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr"/>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>May 2025</t>
+          <t>May 24, 2026</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr">
         <is>
-          <t>Inquired</t>
-        </is>
-      </c>
-      <c r="K8" s="8" t="inlineStr">
-        <is>
-          <t>Rental inquiry via StreetEasy May 2025. Building: The Ashford NYC. Contact Maria Skovranova. Price not confirmed.</t>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Contacted – Awaiting Response</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>StreetEasy inquiry sent May 24, 2026. No broker reply received as of May 25, 2026. Broker name/email TBD.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:L1"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -972,10 +997,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="85" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1029,7 +1054,7 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Example: "Add 123 Main St, Unit 4A, asking $1.2M, purchase, broker Jane Smith at jane@compass.com, showing June 1"</t>
+          <t xml:space="preserve">  Example: "Add 123 Main St, Unit 4A, asking $1.2M, purchase, broker Jane Smith at jane@compass.com, showing June 1 at 2pm"</t>
         </is>
       </c>
     </row>
@@ -1043,105 +1068,147 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Example: "Mark 345 East 80th #27B as Passed"</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
           <t>• Claude reads this file, applies your change, saves, and commits.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>UPLOADING A SCREENSHOT OR EMAIL TO CHECK IF IT'S IN THE LIST</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>• Paste or drag an image / screenshot into the Claude chat.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ask: "Is this apartment already in my tracker?"</t>
+          <t>• Paste or drag an image / screenshot into the Claude chat.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Ask: "Is this apartment already in my tracker?"</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
           <t>• Claude will read the address from the image and search the spreadsheet for a match.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>STATUS KEY</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>• Active – Negotiating  →  offer submitted, back-and-forth in progress</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>• Under Contract        →  agreed price, attorney review / board package stage</t>
+          <t>• Active – Negotiating         →  offer submitted, back-and-forth in progress</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>• Inquired              →  reached out, waiting or toured only</t>
+          <t>• Under Contract               →  agreed price, attorney review / board package stage</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>• Passed                →  decided not to proceed</t>
+          <t>• Showing Scheduled            →  showing confirmed with date &amp; time</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr"/>
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>• Contacted – Scheduling       →  broker replied, arranging showing date</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>ROW COLOUR KEY</t>
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>• Contacted – Awaiting Response →  message sent, no reply yet</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>• Green  →  Purchase listing, active or under contract</t>
+          <t>• Contacted – Circle Back When Ready → broker said to reach out later</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>• Yellow →  Rental listing</t>
+          <t>• Inquired                     →  reached out, waiting or toured only</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>• Passed                       →  decided not to proceed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>ROW COLOUR KEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>• Green  →  Purchase listing, active or under contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>• Yellow →  Rental listing, showing scheduled or inquired</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>• Blue   →  Contacted (rental, awaiting reply or scheduling)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>• Orange →  Passed / no longer pursuing</t>
         </is>

</xml_diff>